<commit_message>
Grow atlas via OpenAlex search: 23 contrasts across 13 studies
Ran systematic search (400 OpenAlex hits; Europe PMC unreachable), auto-screened
with human review of edge cases, and extracted new priming/TGP contrasts.

- Screening: 406 records (13 include / 393 exclude); PRISMA regenerated
- New extractions: Parker OA TGP series, Lafont poly(I:C) maternal priming,
  Griffith costly OA TGP, Putnam/Bellantuono coral preconditioning, plus
  urchin/fish/bryozoan TGP studies
- Flagship bivalve×past-metamorphosis filter now returns 2 contrasts

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/atlas.xlsx
+++ b/data/atlas.xlsx
@@ -12,8 +12,8 @@
     <sheet name="schema" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'atlas'!$A$1:$AT$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'flagship'!$A$1:$AT$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'atlas'!$A$1:$AT$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'flagship'!$A$1:$AT$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'schema'!$A$1:$E$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT8"/>
+  <dimension ref="A1:AT24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2174,8 +2174,3168 @@
       </c>
       <c r="AT8" t="inlineStr"/>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>parker2011-01</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>parker2011</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>10.1111/j.1365-2486.2011.02520.x</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Parker</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Adult OA exposure influences oyster offspring response</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Saccostrea glomerata</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Sydney rock oyster</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>bivalve</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Bivalvia</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>biparental</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>gamete-broodstock</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>veliger-larva</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>adult reproductive conditioning under elevated PCO2</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>OA-low-pH</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>elevated PCO2 during reproductive conditioning</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>elevated PCO2 (OA treatment vs ambient)</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>growth-size</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>larval growth and developmental rate</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>beneficial</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>larvae</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>not-tested</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>positive carryover assayed at larval stage only in this paper</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>adult OA conditioning then offspring reared at elevated/ambient PCO2; wild + selectively bred lines</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr"/>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t>abstract + OpenAlex</t>
+        </is>
+      </c>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>search-extract-v1</t>
+        </is>
+      </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>foundational Sydney rock oyster parental OA priming paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>parker2011-02</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>parker2011</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>10.1111/j.1365-2486.2011.02520.x</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Parker</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Adult OA exposure influences oyster offspring response</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Saccostrea glomerata</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Sydney rock oyster</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>bivalve</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Bivalvia</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>biparental</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>gamete-broodstock</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>veliger-larva</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>adult reproductive conditioning under elevated PCO2</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>OA-low-pH</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>elevated PCO2 during reproductive conditioning</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>elevated PCO2 (OA treatment vs ambient)</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>survival</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>larval survival under elevated PCO2</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>beneficial</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>larvae</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>not-tested</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>adult OA conditioning then offspring reared at elevated/ambient PCO2</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t>abstract + OpenAlex</t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>search-extract-v1</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AT10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>parker2015-01</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>parker2015</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>10.1371/journal.pone.0132276</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Parker</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Persistence of positive OA carryover effects in S. glomerata</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Saccostrea glomerata</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Sydney rock oyster</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>bivalve</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Bivalvia</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>biparental</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>gamete-broodstock</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>transgenerational exposure of adults to elevated CO2; F1 tracked to adulthood</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>OA-low-pH</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>elevated CO2 / ocean acidification</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>elevated CO2 vs ambient</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>physiology-other</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>positive carryover performance into adulthood under OA</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>beneficial</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>F1 adulthood</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>explicit test that larval/juvenile positive carryover persists into adulthood</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>transgenerational OA; F1 followed to adulthood; subsequent generation also tested</t>
+        </is>
+      </c>
+      <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>abstract + OpenAlex</t>
+        </is>
+      </c>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>search-extract-v1</t>
+        </is>
+      </c>
+      <c r="AS11" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t>flagship: bivalve broodstock-primed OA effect persists past metamorphosis into adulthood</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>parker2015-02</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>parker2015</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>10.1371/journal.pone.0132276</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Parker</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Persistence of positive OA carryover effects in S. glomerata</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Saccostrea glomerata</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Sydney rock oyster</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>bivalve</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Bivalvia</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>F0-F1</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>biparental</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>gamete-broodstock</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>spat-juvenile</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>subsequent transgenerational exposure of F1 adults; F2 larvae/juveniles assayed</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>OA-low-pH</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>elevated CO2 / ocean acidification</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>elevated CO2 vs ambient</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>survival</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>F2 larval/juvenile performance under OA</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>beneficial</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr"/>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>F2 larvae/juveniles</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>not-tested</t>
+        </is>
+      </c>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t>tests whether adaptive responses appear in the next generation after F1 adult re-exposure</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK12" t="inlineStr"/>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>multi-generation OA exposure</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr"/>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>abstract + OpenAlex</t>
+        </is>
+      </c>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>search-extract-v1</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AT12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>parker2021-01</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>parker2021</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>10.1242/jeb.239269</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Parker</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Oyster OA TGP differs with intertidal vs subtidal habitat</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Saccostrea glomerata</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Sydney rock oyster</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>bivalve</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Bivalvia</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>biparental</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>gamete-broodstock</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>veliger-larva</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>parental OA exposure under emersion (intertidal) vs continuous immersion (subtidal)</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>OA-low-pH</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>elevated CO2 with/without tidal emersion</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>elevated CO2; habitat = emersion vs immersion</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>physiology-other</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>TGP magnitude/direction depends on parental habitat</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr"/>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>larvae/juveniles</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>not-tested</t>
+        </is>
+      </c>
+      <c r="AI13" t="inlineStr"/>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK13" t="inlineStr"/>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>parental habitat (emersion/immersion) x elevated CO2 TGP design</t>
+        </is>
+      </c>
+      <c r="AO13" t="inlineStr"/>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>abstract + OpenAlex</t>
+        </is>
+      </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>search-extract-v1</t>
+        </is>
+      </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t>shows TGP to OA is habitat-context dependent</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>lafont2018-01</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>lafont2018</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>10.1016/j.dci.2018.09.022</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Lafont</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Maternal poly(I:C) priming improves larval OsHV-1 survival</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Crassostrea gigas</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Pacific oyster</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>bivalve</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Bivalvia</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>maternal</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>gamete-broodstock</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>veliger-larva</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>adult injection of poly(I:C) 3 or 10 days prior to strip-spawning</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>pathogen-immune</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>poly(I:C) viral mimic (OsHV-1 priming)</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>mg/ml</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>100 uL poly(I:C) at 5 mg/ml injected into adductor muscle</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>immune-challenge</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>larval cumulative mortality 48 h post OsHV-1 inoculation</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>beneficial</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>14.4</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>percent-change</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>larvae 48 h post-challenge</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>not-tested</t>
+        </is>
+      </c>
+      <c r="AI14" t="inlineStr">
+        <is>
+          <t>3-day pre-spawn maternal priming reduced larval mortality to 14.4% vs 45.3% control; 10-day priming weaker/ns</t>
+        </is>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK14" t="inlineStr"/>
+      <c r="AL14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AM14" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AN14" t="inlineStr">
+        <is>
+          <t>maternal vs paternal poly(I:C); time-to-spawn factorial; RNA-seq on unchallenged larvae</t>
+        </is>
+      </c>
+      <c r="AO14" t="inlineStr">
+        <is>
+          <t>up to 6 pair-mated families per treatment</t>
+        </is>
+      </c>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>Lafont et al. DCI manuscript methods/results</t>
+        </is>
+      </c>
+      <c r="AQ14" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>search-extract-v1</t>
+        </is>
+      </c>
+      <c r="AS14" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AT14" t="inlineStr">
+        <is>
+          <t>framework Section-6 precedent: poly(I:C) broodstock priming → herpesvirus-resistant offspring</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>lafont2018-02</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>lafont2018</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>10.1016/j.dci.2018.09.022</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Lafont</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Maternal poly(I:C) priming improves larval OsHV-1 survival</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Crassostrea gigas</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Pacific oyster</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>bivalve</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Bivalvia</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>paternal</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>gamete-broodstock</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>veliger-larva</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>paternal poly(I:C) injection prior to spawning</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>pathogen-immune</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>poly(I:C) viral mimic (OsHV-1 priming)</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>mg/ml</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>100 uL poly(I:C) at 5 mg/ml injected into adductor muscle</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>immune-challenge</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>larval survival after OsHV-1 challenge</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr"/>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>larvae</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>not-tested</t>
+        </is>
+      </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>paternal priming had no significant effect; maternal channel only</t>
+        </is>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr"/>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>maternal vs paternal cross design</t>
+        </is>
+      </c>
+      <c r="AO15" t="inlineStr"/>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>Lafont et al. DCI results</t>
+        </is>
+      </c>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>search-extract-v1</t>
+        </is>
+      </c>
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AT15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>lafont2018-03</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>lafont2018</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>10.1016/j.dci.2018.09.022</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Lafont</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Maternal poly(I:C) priming improves larval OsHV-1 survival</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Crassostrea gigas</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Pacific oyster</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>bivalve</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Bivalvia</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>maternal</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>gamete-broodstock</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>veliger-larva</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>adult poly(I:C) prior to spawning</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>pathogen-immune</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>poly(I:C) viral mimic (OsHV-1 priming)</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>mg/ml</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>100 uL poly(I:C) at 5 mg/ml</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>transcriptome</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>antiviral gene expression in unchallenged larvae (RNA-seq)</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr"/>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>unchallenged larvae</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>not-tested</t>
+        </is>
+      </c>
+      <c r="AI16" t="inlineStr">
+        <is>
+          <t>no evidence parental poly(I:C) reconfigures constitutive antiviral transcriptome; maternal provisioning hypothesized</t>
+        </is>
+      </c>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK16" t="inlineStr"/>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>RNA-seq of unchallenged larvae from primed vs control mothers</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr"/>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>Lafont et al. DCI abstract/results</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>search-extract-v1</t>
+        </is>
+      </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AT16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>griffith2017-01</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>griffith2017</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-017-11442-3</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Griffith</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Parental OA makes clam/scallop offspring more vulnerable</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Mercenaria mercenaria</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>hard clam</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>bivalve</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Bivalvia</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>biparental</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>gamete-broodstock</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>veliger-larva</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>adults under high vs low pCO2 during gametogenesis</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>OA-low-pH</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>elevated pCO2 during gametogenesis</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>high vs ambient pCO2</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>survival</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>larval vulnerability to low pH and additional stressors</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>costly</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr"/>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>larvae under low pH + thermal/food/HAB stress</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>not-tested</t>
+        </is>
+      </c>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t>no beneficial TGP; offspring of high-pCO2 adults more vulnerable</t>
+        </is>
+      </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK17" t="inlineStr"/>
+      <c r="AL17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AM17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AN17" t="inlineStr">
+        <is>
+          <t>parental pCO2 x offspring pH x additional stressors</t>
+        </is>
+      </c>
+      <c r="AO17" t="inlineStr"/>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>abstract + OpenAlex</t>
+        </is>
+      </c>
+      <c r="AQ17" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t>search-extract-v1</t>
+        </is>
+      </c>
+      <c r="AS17" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AT17" t="inlineStr">
+        <is>
+          <t>important counterexample: parental OA priming can be maladaptive</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>griffith2017-02</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>griffith2017</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-017-11442-3</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Griffith</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Parental OA makes clam/scallop offspring more vulnerable</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Argopecten irradians</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>bay scallop</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>bivalve</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Bivalvia</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>biparental</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>gamete-broodstock</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>veliger-larva</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>adults under high vs low pCO2 during gametogenesis</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>OA-low-pH</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>elevated pCO2 during gametogenesis</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>high vs ambient pCO2</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>survival</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>larval vulnerability to low pH and additional stressors</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>costly</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr"/>
+      <c r="AF18" t="inlineStr"/>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>larvae</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr">
+        <is>
+          <t>not-tested</t>
+        </is>
+      </c>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK18" t="inlineStr"/>
+      <c r="AL18" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AM18" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AN18" t="inlineStr">
+        <is>
+          <t>parental pCO2 x offspring pH x additional stressors</t>
+        </is>
+      </c>
+      <c r="AO18" t="inlineStr"/>
+      <c r="AP18" t="inlineStr">
+        <is>
+          <t>abstract + OpenAlex</t>
+        </is>
+      </c>
+      <c r="AQ18" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AR18" t="inlineStr">
+        <is>
+          <t>search-extract-v1</t>
+        </is>
+      </c>
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AT18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>putnam2015-01</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>putnam2015</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>10.1242/jeb.123018</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Putnam</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Pocillopora parental temp+OA preconditioning and larval TGP</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Pocillopora damicornis</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>cauliflower coral</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>coral</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Anthozoa</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>maternal</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>veliger-larva</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>adult exposure during larval brooding period</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>multiple</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>elevated temperature + OA (28.9C, 805 uatm PCO2)</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>28.9C + 805 uatm vs ambient 26.5C + 417 uatm</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr"/>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>physiology-other</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>larval performance / parental-effects evidence under future climate</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr"/>
+      <c r="AF19" t="inlineStr"/>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>released larvae</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr">
+        <is>
+          <t>not-tested</t>
+        </is>
+      </c>
+      <c r="AI19" t="inlineStr">
+        <is>
+          <t>adult performance negatively affected; larvae show parental effects (TGP potential)</t>
+        </is>
+      </c>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK19" t="inlineStr"/>
+      <c r="AL19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AM19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AN19" t="inlineStr">
+        <is>
+          <t>adult high vs ambient temp+OA during brooding; larval assays</t>
+        </is>
+      </c>
+      <c r="AO19" t="inlineStr"/>
+      <c r="AP19" t="inlineStr">
+        <is>
+          <t>abstract + OpenAlex</t>
+        </is>
+      </c>
+      <c r="AQ19" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AR19" t="inlineStr">
+        <is>
+          <t>search-extract-v1</t>
+        </is>
+      </c>
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AT19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>bellantuono2011-01</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>bellantuono2011</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>10.1098/rspb.2011.1780</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Bellantuono</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Short-term thermal preconditioning confers coral bleaching resistance</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Acropora millepora</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>staghorn coral</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>coral</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Anthozoa</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>somatic-within-gen</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>10-day preconditioning at 3C below bleaching threshold</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>thermal</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>sub-bleaching thermal preconditioning</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>temperature 3C below experimentally determined bleaching threshold</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>physiology-other</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>symbiosis stability / bleaching resistance under subsequent thermal stress</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>beneficial</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>adult under acute thermal stress</t>
+        </is>
+      </c>
+      <c r="AH20" t="inlineStr"/>
+      <c r="AI20" t="inlineStr">
+        <is>
+          <t>within-generation acquired thermal tolerance; no symbiont community shift</t>
+        </is>
+      </c>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK20" t="inlineStr"/>
+      <c r="AL20" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AM20" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>short-term thermal preconditioning then heat challenge; symbiont/bacterial genotyping</t>
+        </is>
+      </c>
+      <c r="AO20" t="inlineStr"/>
+      <c r="AP20" t="inlineStr">
+        <is>
+          <t>abstract + OpenAlex</t>
+        </is>
+      </c>
+      <c r="AQ20" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AR20" t="inlineStr">
+        <is>
+          <t>search-extract-v1</t>
+        </is>
+      </c>
+      <c r="AS20" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AT20" t="inlineStr">
+        <is>
+          <t>restoration-relevant within-gen thermal hardening</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>clark2019-01</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>clark2019</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-018-37255-6</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Clark</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Molecular mechanisms of low-pH TGP in green sea urchin</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Psammechinus miliaris</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>green sea urchin</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>echinoderm</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Echinoidea</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>biparental</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>embryo</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>adult pre-acclimation to low pH; larvae spawned into low pH</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>OA-low-pH</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>low pH adult preconditioning</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>low pH vs ambient</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>transcriptome</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>larval RNA-seq; antioxidant pre-loading signature</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>beneficial</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr"/>
+      <c r="AF21" t="inlineStr"/>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>larvae under low pH</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr">
+        <is>
+          <t>not-tested</t>
+        </is>
+      </c>
+      <c r="AI21" t="inlineStr">
+        <is>
+          <t>adult conditioning pre-loads embryonic transcriptional pool with antioxidants</t>
+        </is>
+      </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK21" t="inlineStr"/>
+      <c r="AL21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AM21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>adult low-pH acclimation then offspring RNA-seq under low pH</t>
+        </is>
+      </c>
+      <c r="AO21" t="inlineStr"/>
+      <c r="AP21" t="inlineStr">
+        <is>
+          <t>abstract + OpenAlex</t>
+        </is>
+      </c>
+      <c r="AQ21" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AR21" t="inlineStr">
+        <is>
+          <t>search-extract-v1</t>
+        </is>
+      </c>
+      <c r="AS21" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AT21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>donelson2016-01</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>donelson2016</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>10.1111/eva.12386</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Donelson</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Gradual warming across generations improves reproductive TGP</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Acanthochromis polyacanthus</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>spiny chromis</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>fish</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Actinopterygii</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>F0-F1</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>biparental</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>whole-lifecycle</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>+1.5C in F0 then +3.0C in F1 (gradual) vs abrupt warming</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>thermal</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>ocean warming across generations</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>+1.5C then +3.0C vs controls/abrupt</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>reproduction</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>reproductive output and offspring quality</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>beneficial</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr"/>
+      <c r="AF22" t="inlineStr"/>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>F1 adults / their offspring</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr"/>
+      <c r="AI22" t="inlineStr">
+        <is>
+          <t>gradual warming over two generations yielded greater reproductive plasticity than abrupt</t>
+        </is>
+      </c>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK22" t="inlineStr"/>
+      <c r="AL22" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AM22" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AN22" t="inlineStr">
+        <is>
+          <t>multi-generation thermal acclimation rate experiment</t>
+        </is>
+      </c>
+      <c r="AO22" t="inlineStr"/>
+      <c r="AP22" t="inlineStr">
+        <is>
+          <t>abstract + OpenAlex</t>
+        </is>
+      </c>
+      <c r="AQ22" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AR22" t="inlineStr">
+        <is>
+          <t>search-extract-v1</t>
+        </is>
+      </c>
+      <c r="AS22" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AT22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>shama2014-01</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>shama2014</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>10.1111/1365-2435.12280</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Shama</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Maternal TGP mediates stickleback offspring size under warming</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Gasterosteus aculeatus</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>three-spined stickleback</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>fish</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Actinopterygii</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>maternal</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>spat-juvenile</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>maternal acclimation to 17C or 21C; offspring reared at matching/mismatching temps</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>thermal</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>maternal warming acclimation</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>degC</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>maternal 17C vs 21C; offspring cross-factored</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr"/>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>growth-size</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>offspring body size to 30 days (and beyond)</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>beneficial</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>offspring &gt;=30 days</t>
+        </is>
+      </c>
+      <c r="AH23" t="inlineStr"/>
+      <c r="AI23" t="inlineStr">
+        <is>
+          <t>maternal TGP benefits on size stronger/longer under warmer conditions</t>
+        </is>
+      </c>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK23" t="inlineStr"/>
+      <c r="AL23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AM23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AN23" t="inlineStr">
+        <is>
+          <t>TGP x quantitative genetics; mitochondrial respiration mechanism</t>
+        </is>
+      </c>
+      <c r="AO23" t="inlineStr"/>
+      <c r="AP23" t="inlineStr">
+        <is>
+          <t>abstract + OpenAlex</t>
+        </is>
+      </c>
+      <c r="AQ23" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AR23" t="inlineStr">
+        <is>
+          <t>search-extract-v1</t>
+        </is>
+      </c>
+      <c r="AS23" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AT23" t="inlineStr">
+        <is>
+          <t>marine stickleback population</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>marshall2008-01</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>marshall2008</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>10.1890/07-0449.1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Marshall</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Context-dependent maternal copper effects across life history</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Bugula neritina</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>brown bryozoan</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Gymnolaemata</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>maternal</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>whole-lifecycle</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>maternal colonies exposed to copper pollution stress in lab</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>pollutant</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>copper</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>copper exposure of maternal colonies</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>survival</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>offspring performance across life-history stages (context-dependent)</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr"/>
+      <c r="AF24" t="inlineStr"/>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>multiple post-settlement stages</t>
+        </is>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AI24" t="inlineStr">
+        <is>
+          <t>maternal effects can increase performance in one stage and reduce it in another; assayed across life history incl. post-metamorphosis</t>
+        </is>
+      </c>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK24" t="inlineStr"/>
+      <c r="AL24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AM24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AN24" t="inlineStr">
+        <is>
+          <t>maternal copper exposure; offspring tracked across life history</t>
+        </is>
+      </c>
+      <c r="AO24" t="inlineStr"/>
+      <c r="AP24" t="inlineStr">
+        <is>
+          <t>abstract + OpenAlex</t>
+        </is>
+      </c>
+      <c r="AQ24" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>search-extract-v1</t>
+        </is>
+      </c>
+      <c r="AS24" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AT24" t="inlineStr">
+        <is>
+          <t>classic marine TGP / maternal-effects paper; taxon_group=other (bryozoan)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AT8"/>
+  <autoFilter ref="A1:AT24"/>
   <dataValidations count="20">
     <dataValidation sqref="I2:I2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"bivalve,coral,fish,gastropod,crustacean,echinoderm,cephalopod,macroalgae,other,NA,NR"</formula1>
@@ -2248,7 +5408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT2"/>
+  <dimension ref="A1:AT3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2699,8 +5859,204 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>parker2015-01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>parker2015</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>10.1371/journal.pone.0132276</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Parker</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Persistence of positive OA carryover effects in S. glomerata</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Saccostrea glomerata</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Sydney rock oyster</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>bivalve</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Bivalvia</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>biparental</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>gamete-broodstock</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>transgenerational exposure of adults to elevated CO2; F1 tracked to adulthood</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>OA-low-pH</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>elevated CO2 / ocean acidification</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>elevated CO2 vs ambient</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>physiology-other</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>positive carryover performance into adulthood under OA</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>beneficial</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>F1 adulthood</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>explicit test that larval/juvenile positive carryover persists into adulthood</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>transgenerational OA; F1 followed to adulthood; subsequent generation also tested</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>abstract + OpenAlex</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>search-extract-v1</t>
+        </is>
+      </c>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>flagship: bivalve broodstock-primed OA effect persists past metamorphosis into adulthood</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AT2"/>
+  <autoFilter ref="A1:AT3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Correct atlas extraction errors for DOIs, species, and priming life stages.
Source-check carryover/TGP rows (Spencer, Alma, Pereira, Gurr, Hettinger) and fill the Sol Dourdin DOI so generation and life-stage coding match the primary literature.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/atlas.xlsx
+++ b/data/atlas.xlsx
@@ -727,7 +727,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>NR</t>
+          <t>10.1021/acs.est.3c08201</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>NR</t>
+          <t>10.1021/acs.est.3c08201</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>NR</t>
+          <t>10.1021/acs.est.3c08201</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>NR</t>
+          <t>10.1021/acs.est.3c08201</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -6360,11 +6360,7 @@
       <c r="AE30" t="inlineStr"/>
       <c r="AF30" t="inlineStr"/>
       <c r="AG30" t="inlineStr"/>
-      <c r="AH30" t="inlineStr">
-        <is>
-          <t>not-tested</t>
-        </is>
-      </c>
+      <c r="AH30" t="inlineStr"/>
       <c r="AI30" t="inlineStr"/>
       <c r="AJ30" t="inlineStr">
         <is>
@@ -10047,7 +10043,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>10.1111/gcb.12293</t>
+          <t>10.1111/gcb.12307</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -10137,12 +10133,12 @@
       </c>
       <c r="Y51" t="inlineStr">
         <is>
-          <t>survival</t>
+          <t>growth-size</t>
         </is>
       </c>
       <c r="Z51" t="inlineStr">
         <is>
-          <t>field juvenile performance after larval OA</t>
+          <t>field juvenile growth after larval OA (carryover unabated 4 months)</t>
         </is>
       </c>
       <c r="AA51" t="inlineStr">
@@ -10165,7 +10161,7 @@
       <c r="AF51" t="inlineStr"/>
       <c r="AG51" t="inlineStr">
         <is>
-          <t>field juveniles</t>
+          <t>field juveniles 4 months post-outplant</t>
         </is>
       </c>
       <c r="AH51" t="inlineStr">
@@ -10175,7 +10171,7 @@
       </c>
       <c r="AI51" t="inlineStr">
         <is>
-          <t>carryover persists under natural environmental conditions</t>
+          <t>larval pCO2 carryover on growth persists in field; juvenile survival driven by shore level not larval pCO2</t>
         </is>
       </c>
       <c r="AJ51" t="inlineStr">
@@ -10196,13 +10192,13 @@
       </c>
       <c r="AN51" t="inlineStr">
         <is>
-          <t>lab larval OA then field deployment</t>
+          <t>lab larval OA then field deployment mid/low intertidal</t>
         </is>
       </c>
       <c r="AO51" t="inlineStr"/>
       <c r="AP51" t="inlineStr">
         <is>
-          <t>user bibliography + title/abstract</t>
+          <t>abstract + full text (10.1111/gcb.12307)</t>
         </is>
       </c>
       <c r="AQ51" t="inlineStr">
@@ -10220,7 +10216,11 @@
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="AT51" t="inlineStr"/>
+      <c r="AT51" t="inlineStr">
+        <is>
+          <t>corrected 2026-08-04: DOI was 10.1111/gcb.12293 (typo); assay is growth carryover not survival</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -10280,17 +10280,17 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>somatic-within-gen</t>
+          <t>biparental</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>veliger-larva</t>
+          <t>adult</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
@@ -10300,7 +10300,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>early-life temperature and pCO2 treatments across populations</t>
+          <t>adult parental exposure to elevated winter temperature (+4C) then elevated pCO2 during reproductive conditioning</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
@@ -10310,12 +10310,16 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>temperature + elevated pCO2</t>
+          <t>elevated winter temperature + pCO2</t>
         </is>
       </c>
       <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr"/>
-      <c r="U52" t="inlineStr"/>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>+4C (at 10C); +2204 uatm pCO2 (at 3045 uatm)</t>
+        </is>
+      </c>
       <c r="V52" t="inlineStr"/>
       <c r="W52" t="inlineStr"/>
       <c r="X52" t="inlineStr">
@@ -10325,12 +10329,12 @@
       </c>
       <c r="Y52" t="inlineStr">
         <is>
-          <t>growth-size</t>
+          <t>survival</t>
         </is>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
-          <t>carryover effects on later performance across populations</t>
+          <t>offspring field survival after parental exposure (higher in 2 of 4 bays)</t>
         </is>
       </c>
       <c r="AA52" t="inlineStr">
@@ -10353,7 +10357,7 @@
       <c r="AF52" t="inlineStr"/>
       <c r="AG52" t="inlineStr">
         <is>
-          <t>juveniles</t>
+          <t>offspring juveniles outplanted to 4 bays</t>
         </is>
       </c>
       <c r="AH52" t="inlineStr">
@@ -10361,7 +10365,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AI52" t="inlineStr"/>
+      <c r="AI52" t="inlineStr">
+        <is>
+          <t>effect detected in post-metamorphic offspring after ~1 yr common-garden + 3 mo field</t>
+        </is>
+      </c>
       <c r="AJ52" t="inlineStr">
         <is>
           <t>no</t>
@@ -10380,18 +10388,18 @@
       </c>
       <c r="AN52" t="inlineStr">
         <is>
-          <t>multi-population developmental carryover</t>
+          <t>parental temp+pCO2 exposure; F1 reared ~1 yr then outplanted to 4 estuarine bays</t>
         </is>
       </c>
       <c r="AO52" t="inlineStr"/>
       <c r="AP52" t="inlineStr">
         <is>
-          <t>user bibliography + title/abstract</t>
+          <t>abstract + full text (10.1002/eap.2060)</t>
         </is>
       </c>
       <c r="AQ52" t="inlineStr">
         <is>
-          <t>med</t>
+          <t>high</t>
         </is>
       </c>
       <c r="AR52" t="inlineStr">
@@ -10404,7 +10412,11 @@
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="AT52" t="inlineStr"/>
+      <c r="AT52" t="inlineStr">
+        <is>
+          <t>corrected 2026-08-04: parents primed as ADULTS; intergenerational F0-&gt;F1 carryover (was mis-coded within-gen larval)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -10439,12 +10451,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Saccostrea glomerata</t>
+          <t>Ostrea angasi</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Sydney rock oyster</t>
+          <t>Australian flat oyster</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -10474,17 +10486,17 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>spat-juvenile</t>
+          <t>adult</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>spat-juvenile</t>
+          <t>adult</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>prior stress exposure then ocean warming challenge</t>
+          <t>adult laboratory heat shock then field ocean-warming proxy</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
@@ -10494,14 +10506,14 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>prior stress priming for warming</t>
+          <t>prior heat-shock priming for warming</t>
         </is>
       </c>
       <c r="S53" t="inlineStr"/>
       <c r="T53" t="inlineStr"/>
       <c r="U53" t="inlineStr">
         <is>
-          <t>prior stress then warming; two oyster species</t>
+          <t>lab heat shock then power-plant thermal outfall field exposure</t>
         </is>
       </c>
       <c r="V53" t="inlineStr"/>
@@ -10518,7 +10530,7 @@
       </c>
       <c r="Z53" t="inlineStr">
         <is>
-          <t>resilience to ocean warming after prior stress</t>
+          <t>survival under ocean warming after prior heat shock</t>
         </is>
       </c>
       <c r="AA53" t="inlineStr">
@@ -10539,9 +10551,17 @@
       </c>
       <c r="AE53" t="inlineStr"/>
       <c r="AF53" t="inlineStr"/>
-      <c r="AG53" t="inlineStr"/>
+      <c r="AG53" t="inlineStr">
+        <is>
+          <t>adults in field warming proxy</t>
+        </is>
+      </c>
       <c r="AH53" t="inlineStr"/>
-      <c r="AI53" t="inlineStr"/>
+      <c r="AI53" t="inlineStr">
+        <is>
+          <t>within-generation adult hardening; heat shock did little overall but improved O. angasi survival</t>
+        </is>
+      </c>
       <c r="AJ53" t="inlineStr">
         <is>
           <t>no</t>
@@ -10560,18 +10580,18 @@
       </c>
       <c r="AN53" t="inlineStr">
         <is>
-          <t>prior stress x warming; two species</t>
+          <t>adult heat shock then field warming; also assayed Saccostrea glomerata</t>
         </is>
       </c>
       <c r="AO53" t="inlineStr"/>
       <c r="AP53" t="inlineStr">
         <is>
-          <t>user bibliography + title/abstract</t>
+          <t>abstract + full text (10.1371/journal.pone.0228527)</t>
         </is>
       </c>
       <c r="AQ53" t="inlineStr">
         <is>
-          <t>med</t>
+          <t>high</t>
         </is>
       </c>
       <c r="AR53" t="inlineStr">
@@ -10586,7 +10606,7 @@
       </c>
       <c r="AT53" t="inlineStr">
         <is>
-          <t>also includes a second oyster species in the paper</t>
+          <t>corrected 2026-08-04: primed as ADULTS not spat; primary survival benefit in O. angasi (also tested S. glomerata)</t>
         </is>
       </c>
     </row>
@@ -10623,12 +10643,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Leukoma staminea</t>
+          <t>Panopea generosa</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Pacific littleneck clam</t>
+          <t>Pacific geoduck</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -10658,17 +10678,17 @@
       </c>
       <c r="N54" t="inlineStr">
         <is>
+          <t>pediveliger-larva</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
           <t>spat-juvenile</t>
         </is>
       </c>
-      <c r="O54" t="inlineStr">
-        <is>
-          <t>spat-juvenile</t>
-        </is>
-      </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>repeat exposure to hypercapnic seawater</t>
+          <t>pediveliger conditioned 110 days under moderate pCO2 then repeat exposures</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -10683,9 +10703,21 @@
       </c>
       <c r="S54" t="inlineStr"/>
       <c r="T54" t="inlineStr"/>
-      <c r="U54" t="inlineStr"/>
-      <c r="V54" t="inlineStr"/>
-      <c r="W54" t="inlineStr"/>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>ambient ~920 uatm vs moderate ~2800 uatm then severe/moderate re-exposures</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
       <c r="X54" t="inlineStr">
         <is>
           <t>yes</t>
@@ -10698,12 +10730,12 @@
       </c>
       <c r="Z54" t="inlineStr">
         <is>
-          <t>growth and oxidative status after repeated hypercapnia</t>
+          <t>respiration organic biomass shell size and antioxidant capacity after repeated hypercapnia</t>
         </is>
       </c>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>beneficial</t>
         </is>
       </c>
       <c r="AB54" t="inlineStr"/>
@@ -10719,9 +10751,21 @@
       </c>
       <c r="AE54" t="inlineStr"/>
       <c r="AF54" t="inlineStr"/>
-      <c r="AG54" t="inlineStr"/>
-      <c r="AH54" t="inlineStr"/>
-      <c r="AI54" t="inlineStr"/>
+      <c r="AG54" t="inlineStr">
+        <is>
+          <t>juveniles after secondary/tertiary exposures</t>
+        </is>
+      </c>
+      <c r="AH54" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AI54" t="inlineStr">
+        <is>
+          <t>initial pediveliger conditioning effects assayed in juveniles past metamorphosis</t>
+        </is>
+      </c>
       <c r="AJ54" t="inlineStr">
         <is>
           <t>no</t>
@@ -10740,18 +10784,18 @@
       </c>
       <c r="AN54" t="inlineStr">
         <is>
-          <t>repeat vs single hypercapnia exposure</t>
+          <t>pediveliger-to-juvenile pCO2 conditioning with reciprocal re-exposures</t>
         </is>
       </c>
       <c r="AO54" t="inlineStr"/>
       <c r="AP54" t="inlineStr">
         <is>
-          <t>user bibliography + title/abstract</t>
+          <t>abstract + full text (10.1242/jeb.233932)</t>
         </is>
       </c>
       <c r="AQ54" t="inlineStr">
         <is>
-          <t>med</t>
+          <t>high</t>
         </is>
       </c>
       <c r="AR54" t="inlineStr">
@@ -10766,7 +10810,7 @@
       </c>
       <c r="AT54" t="inlineStr">
         <is>
-          <t>confirm species on full text if needed</t>
+          <t>corrected 2026-08-04: species was mis-coded Leukoma staminea; primed as pediveliger not spat</t>
         </is>
       </c>
     </row>
@@ -11359,12 +11403,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>NR</t>
+          <t>Ostrea lurida</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>NR</t>
+          <t>Olympia oyster</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -11384,27 +11428,27 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>somatic-within-gen</t>
+          <t>biparental</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
         <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
           <t>veliger-larva</t>
         </is>
       </c>
-      <c r="O58" t="inlineStr">
-        <is>
-          <t>spat-juvenile</t>
-        </is>
-      </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>changing-environment exposures with carryover assays</t>
+          <t>adult field acclimatization at Puget Sound buoy sites then spawn</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
@@ -11414,7 +11458,7 @@
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>changing environments (plasticity + carryover)</t>
+          <t>site-specific parental environments (temp/pH/etc)</t>
         </is>
       </c>
       <c r="S58" t="inlineStr"/>
@@ -11434,7 +11478,7 @@
       </c>
       <c r="Z58" t="inlineStr">
         <is>
-          <t>phenotypic plasticity and carryover effects</t>
+          <t>offspring larval survival growth and metabolism under thermal stress</t>
         </is>
       </c>
       <c r="AA58" t="inlineStr">
@@ -11455,13 +11499,21 @@
       </c>
       <c r="AE58" t="inlineStr"/>
       <c r="AF58" t="inlineStr"/>
-      <c r="AG58" t="inlineStr"/>
+      <c r="AG58" t="inlineStr">
+        <is>
+          <t>released larvae under thermal assays</t>
+        </is>
+      </c>
       <c r="AH58" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AI58" t="inlineStr"/>
+          <t>not-tested</t>
+        </is>
+      </c>
+      <c r="AI58" t="inlineStr">
+        <is>
+          <t>parental site history (esp. Dabob Bay) affects larval performance; not assayed past metamorphosis</t>
+        </is>
+      </c>
       <c r="AJ58" t="inlineStr">
         <is>
           <t>no</t>
@@ -11480,18 +11532,18 @@
       </c>
       <c r="AN58" t="inlineStr">
         <is>
-          <t>environmental change with carryover design</t>
+          <t>parental field outplant acclimatization; F1 larval thermal assays</t>
         </is>
       </c>
       <c r="AO58" t="inlineStr"/>
       <c r="AP58" t="inlineStr">
         <is>
-          <t>user bibliography + title/abstract</t>
+          <t>abstract + full text (10.3389/fmars.2024.1178507)</t>
         </is>
       </c>
       <c r="AQ58" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="AR58" t="inlineStr">
@@ -11506,7 +11558,7 @@
       </c>
       <c r="AT58" t="inlineStr">
         <is>
-          <t>species to confirm on full text (Front. Mar. Sci. 2024)</t>
+          <t>corrected 2026-08-04: Ostrea lurida; parents primed as ADULTS (F0-&gt;F1) not within-gen larval</t>
         </is>
       </c>
     </row>
@@ -12787,7 +12839,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>10.1101/773481</t>
+          <t>10.1093/conphys/coaa024</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -12797,7 +12849,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -12852,7 +12904,7 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>short-term acidified seawater then recovery</t>
+          <t>juvenile short-term elevated pCO2 then ambient recovery</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
@@ -12867,9 +12919,21 @@
       </c>
       <c r="S66" t="inlineStr"/>
       <c r="T66" t="inlineStr"/>
-      <c r="U66" t="inlineStr"/>
-      <c r="V66" t="inlineStr"/>
-      <c r="W66" t="inlineStr"/>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>~550 vs ~2400 uatm; 10-day then 6-day reciprocal exposures</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
       <c r="X66" t="inlineStr">
         <is>
           <t>yes</t>
@@ -12882,7 +12946,7 @@
       </c>
       <c r="Z66" t="inlineStr">
         <is>
-          <t>metabolic recovery and compensatory shell growth</t>
+          <t>metabolic recovery and compensatory shell growth (+5.8% shell length at 5 months)</t>
         </is>
       </c>
       <c r="AA66" t="inlineStr">
@@ -12901,11 +12965,27 @@
           <t>sig</t>
         </is>
       </c>
-      <c r="AE66" t="inlineStr"/>
-      <c r="AF66" t="inlineStr"/>
-      <c r="AG66" t="inlineStr"/>
+      <c r="AE66" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AF66" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="AG66" t="inlineStr">
+        <is>
+          <t>5 months post-exposure ambient common garden</t>
+        </is>
+      </c>
       <c r="AH66" t="inlineStr"/>
-      <c r="AI66" t="inlineStr"/>
+      <c r="AI66" t="inlineStr">
+        <is>
+          <t>within-generation juvenile conditioning; no metamorphic transition in design</t>
+        </is>
+      </c>
       <c r="AJ66" t="inlineStr">
         <is>
           <t>no</t>
@@ -12930,12 +13010,12 @@
       <c r="AO66" t="inlineStr"/>
       <c r="AP66" t="inlineStr">
         <is>
-          <t>user bibliography + title/abstract</t>
+          <t>abstract + full text (10.1093/conphys/coaa024)</t>
         </is>
       </c>
       <c r="AQ66" t="inlineStr">
         <is>
-          <t>med</t>
+          <t>high</t>
         </is>
       </c>
       <c r="AR66" t="inlineStr">
@@ -12950,7 +13030,7 @@
       </c>
       <c r="AT66" t="inlineStr">
         <is>
-          <t>bioRxiv preprint</t>
+          <t>corrected 2026-08-04: DOI was wrong bioRxiv 773481; published Conserv Physiol 2020 (preprint 10.1101/689745)</t>
         </is>
       </c>
     </row>
@@ -13456,7 +13536,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>NR</t>
+          <t>10.1021/acs.est.3c08201</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -14252,7 +14332,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>10.1111/gcb.12293</t>
+          <t>10.1111/gcb.12307</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -14342,12 +14422,12 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>survival</t>
+          <t>growth-size</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>field juvenile performance after larval OA</t>
+          <t>field juvenile growth after larval OA (carryover unabated 4 months)</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
@@ -14370,7 +14450,7 @@
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>field juveniles</t>
+          <t>field juveniles 4 months post-outplant</t>
         </is>
       </c>
       <c r="AH6" t="inlineStr">
@@ -14380,7 +14460,7 @@
       </c>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>carryover persists under natural environmental conditions</t>
+          <t>larval pCO2 carryover on growth persists in field; juvenile survival driven by shore level not larval pCO2</t>
         </is>
       </c>
       <c r="AJ6" t="inlineStr">
@@ -14401,13 +14481,13 @@
       </c>
       <c r="AN6" t="inlineStr">
         <is>
-          <t>lab larval OA then field deployment</t>
+          <t>lab larval OA then field deployment mid/low intertidal</t>
         </is>
       </c>
       <c r="AO6" t="inlineStr"/>
       <c r="AP6" t="inlineStr">
         <is>
-          <t>user bibliography + title/abstract</t>
+          <t>abstract + full text (10.1111/gcb.12307)</t>
         </is>
       </c>
       <c r="AQ6" t="inlineStr">
@@ -14425,7 +14505,11 @@
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="AT6" t="inlineStr"/>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>corrected 2026-08-04: DOI was 10.1111/gcb.12293 (typo); assay is growth carryover not survival</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -14485,17 +14569,17 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>somatic-within-gen</t>
+          <t>biparental</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>veliger-larva</t>
+          <t>adult</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -14505,7 +14589,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>early-life temperature and pCO2 treatments across populations</t>
+          <t>adult parental exposure to elevated winter temperature (+4C) then elevated pCO2 during reproductive conditioning</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -14515,12 +14599,16 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>temperature + elevated pCO2</t>
+          <t>elevated winter temperature + pCO2</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>+4C (at 10C); +2204 uatm pCO2 (at 3045 uatm)</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr">
@@ -14530,12 +14618,12 @@
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>growth-size</t>
+          <t>survival</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>carryover effects on later performance across populations</t>
+          <t>offspring field survival after parental exposure (higher in 2 of 4 bays)</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
@@ -14558,7 +14646,7 @@
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>juveniles</t>
+          <t>offspring juveniles outplanted to 4 bays</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr">
@@ -14566,7 +14654,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AI7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>effect detected in post-metamorphic offspring after ~1 yr common-garden + 3 mo field</t>
+        </is>
+      </c>
       <c r="AJ7" t="inlineStr">
         <is>
           <t>no</t>
@@ -14585,18 +14677,18 @@
       </c>
       <c r="AN7" t="inlineStr">
         <is>
-          <t>multi-population developmental carryover</t>
+          <t>parental temp+pCO2 exposure; F1 reared ~1 yr then outplanted to 4 estuarine bays</t>
         </is>
       </c>
       <c r="AO7" t="inlineStr"/>
       <c r="AP7" t="inlineStr">
         <is>
-          <t>user bibliography + title/abstract</t>
+          <t>abstract + full text (10.1002/eap.2060)</t>
         </is>
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>med</t>
+          <t>high</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
@@ -14609,47 +14701,51 @@
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="AT7" t="inlineStr"/>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>corrected 2026-08-04: parents primed as ADULTS; intergenerational F0-&gt;F1 carryover (was mis-coded within-gen larval)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>rondon2017-01</t>
+          <t>gurr2021-01</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>rondon2017</t>
+          <t>gurr2021</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10.1093/eep/dvx004</t>
+          <t>10.1242/jeb.233932</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Rondon</t>
+          <t>Gurr</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Parental diuron exposure alters Pacific oyster spat methylome</t>
+          <t>Repeat hypercapnia modifies growth/oxidative status in burrowing clam</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Crassostrea gigas</t>
+          <t>Panopea generosa</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Pacific oyster</t>
+          <t>Pacific geoduck</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -14669,17 +14765,17 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F0</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>biparental</t>
+          <t>somatic-within-gen</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>gamete-broodstock</t>
+          <t>pediveliger-larva</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -14689,24 +14785,36 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>parental diuron exposure; spat methylome assayed</t>
+          <t>pediveliger conditioned 110 days under moderate pCO2 then repeat exposures</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>pollutant</t>
+          <t>OA-low-pH</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>diuron</t>
+          <t>repeat hypercapnia</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>ambient ~920 uatm vs moderate ~2800 uatm then severe/moderate re-exposures</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
       <c r="X8" t="inlineStr">
         <is>
           <t>yes</t>
@@ -14714,17 +14822,17 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>methylation</t>
+          <t>growth-size</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>F1 spat methylome shifts after parental diuron</t>
+          <t>respiration organic biomass shell size and antioxidant capacity after repeated hypercapnia</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>beneficial</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr"/>
@@ -14742,7 +14850,7 @@
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>spat</t>
+          <t>juveniles after secondary/tertiary exposures</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr">
@@ -14752,19 +14860,15 @@
       </c>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>parental exposure signature detected in post-metamorphic spat methylome</t>
+          <t>initial pediveliger conditioning effects assayed in juveniles past metamorphosis</t>
         </is>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AK8" t="inlineStr">
-        <is>
-          <t>RRBS-Methyl-seq</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr"/>
       <c r="AL8" t="inlineStr">
         <is>
           <t>no</t>
@@ -14777,18 +14881,18 @@
       </c>
       <c r="AN8" t="inlineStr">
         <is>
-          <t>parental pollutant exposure; F1 methylome</t>
+          <t>pediveliger-to-juvenile pCO2 conditioning with reciprocal re-exposures</t>
         </is>
       </c>
       <c r="AO8" t="inlineStr"/>
       <c r="AP8" t="inlineStr">
         <is>
-          <t>user bibliography + title/abstract</t>
+          <t>abstract + full text (10.1242/jeb.233932)</t>
         </is>
       </c>
       <c r="AQ8" t="inlineStr">
         <is>
-          <t>med</t>
+          <t>high</t>
         </is>
       </c>
       <c r="AR8" t="inlineStr">
@@ -14801,47 +14905,51 @@
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="AT8" t="inlineStr"/>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>corrected 2026-08-04: species was mis-coded Leukoma staminea; primed as pediveliger not spat</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>alma2024-01</t>
+          <t>rondon2017-01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>alma2024</t>
+          <t>rondon2017</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.3389/fmars.2024.1178507</t>
+          <t>10.1093/eep/dvx004</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Alma</t>
+          <t>Rondon</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Phenotypic plasticity and carryover in an ecologically important bivalve</t>
+          <t>Parental diuron exposure alters Pacific oyster spat methylome</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>NR</t>
+          <t>Crassostrea gigas</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NR</t>
+          <t>Pacific oyster</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -14861,17 +14969,17 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>F0</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>somatic-within-gen</t>
+          <t>biparental</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>veliger-larva</t>
+          <t>gamete-broodstock</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -14881,17 +14989,17 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>changing-environment exposures with carryover assays</t>
+          <t>parental diuron exposure; spat methylome assayed</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>multiple</t>
+          <t>pollutant</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>changing environments (plasticity + carryover)</t>
+          <t>diuron</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
@@ -14906,12 +15014,12 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>physiology-other</t>
+          <t>methylation</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>phenotypic plasticity and carryover effects</t>
+          <t>F1 spat methylome shifts after parental diuron</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
@@ -14932,19 +15040,31 @@
       </c>
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr"/>
-      <c r="AG9" t="inlineStr"/>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>spat</t>
+        </is>
+      </c>
       <c r="AH9" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="AI9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>parental exposure signature detected in post-metamorphic spat methylome</t>
+        </is>
+      </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AK9" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>RRBS-Methyl-seq</t>
+        </is>
+      </c>
       <c r="AL9" t="inlineStr">
         <is>
           <t>no</t>
@@ -14957,7 +15077,7 @@
       </c>
       <c r="AN9" t="inlineStr">
         <is>
-          <t>environmental change with carryover design</t>
+          <t>parental pollutant exposure; F1 methylome</t>
         </is>
       </c>
       <c r="AO9" t="inlineStr"/>
@@ -14968,7 +15088,7 @@
       </c>
       <c r="AQ9" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>med</t>
         </is>
       </c>
       <c r="AR9" t="inlineStr">
@@ -14981,11 +15101,7 @@
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="AT9" t="inlineStr">
-        <is>
-          <t>species to confirm on full text (Front. Mar. Sci. 2024)</t>
-        </is>
-      </c>
+      <c r="AT9" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AT9"/>

</xml_diff>